<commit_message>
cohens_d and hedges_g (effectsize) In R Software
</commit_message>
<xml_diff>
--- a/effectsize/effectsize.xlsx
+++ b/effectsize/effectsize.xlsx
@@ -413,7 +413,7 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="2">
-        <v>10.819599999999999</v>
+        <v>0</v>
       </c>
       <c r="B2" s="2">
         <v>10.6974</v>
@@ -427,7 +427,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="2">
-        <v>11.0627</v>
+        <v>0</v>
       </c>
       <c r="B3" s="2">
         <v>10.7334</v>
@@ -441,7 +441,7 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="2">
-        <v>11.0627</v>
+        <v>1</v>
       </c>
       <c r="B4" s="2">
         <v>10.7334</v>
@@ -455,7 +455,7 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="2">
-        <v>10.4267</v>
+        <v>0</v>
       </c>
       <c r="B5" s="2">
         <v>10.6135</v>
@@ -469,7 +469,7 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="2">
-        <v>10.6356</v>
+        <v>1</v>
       </c>
       <c r="B6" s="2">
         <v>10.6311</v>
@@ -483,7 +483,7 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="2">
-        <v>10.9838</v>
+        <v>0</v>
       </c>
       <c r="B7" s="2">
         <v>10.644399999999999</v>
@@ -497,7 +497,7 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="2">
-        <v>10.7317</v>
+        <v>0</v>
       </c>
       <c r="B8" s="2">
         <v>11.064399999999999</v>
@@ -511,7 +511,7 @@
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="2">
-        <v>10.972300000000001</v>
+        <v>1</v>
       </c>
       <c r="B9" s="2">
         <v>10.9758</v>
@@ -525,7 +525,7 @@
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="2">
-        <v>10.9925</v>
+        <v>1</v>
       </c>
       <c r="B10" s="2">
         <v>10.9322</v>
@@ -539,7 +539,7 @@
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="2">
-        <v>9.6292000000000009</v>
+        <v>0</v>
       </c>
       <c r="B11" s="2">
         <v>10.6518</v>
@@ -553,7 +553,7 @@
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="2">
-        <v>10.622199999999999</v>
+        <v>0</v>
       </c>
       <c r="B12" s="2">
         <v>10.5532</v>
@@ -567,7 +567,7 @@
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="2">
-        <v>10.7254</v>
+        <v>0</v>
       </c>
       <c r="B13" s="2">
         <v>10.593</v>
@@ -581,7 +581,7 @@
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="2">
-        <v>10.610200000000001</v>
+        <v>1</v>
       </c>
       <c r="B14" s="2">
         <v>10.7478</v>
@@ -595,7 +595,7 @@
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="2">
-        <v>10.6518</v>
+        <v>1</v>
       </c>
       <c r="B15" s="2">
         <v>10.672499999999999</v>
@@ -609,7 +609,7 @@
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="2">
-        <v>10.745200000000001</v>
+        <v>0</v>
       </c>
       <c r="B16" s="2">
         <v>10.666700000000001</v>
@@ -623,7 +623,7 @@
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="2">
-        <v>10.8725</v>
+        <v>0</v>
       </c>
       <c r="B17" s="2">
         <v>10.9207</v>
@@ -637,7 +637,7 @@
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="2">
-        <v>11.0184</v>
+        <v>1</v>
       </c>
       <c r="B18" s="2">
         <v>10.7789</v>
@@ -651,7 +651,7 @@
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="2">
-        <v>11.0665</v>
+        <v>1</v>
       </c>
       <c r="B19" s="2">
         <v>10.81</v>
@@ -665,7 +665,7 @@
     </row>
     <row r="20" spans="1:4">
       <c r="A20" s="2">
-        <v>10.571899999999999</v>
+        <v>0</v>
       </c>
       <c r="B20" s="2">
         <v>10.711</v>
@@ -679,7 +679,7 @@
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="2">
-        <v>10.821999999999999</v>
+        <v>0</v>
       </c>
       <c r="B21" s="2">
         <v>10.6639</v>
@@ -693,7 +693,7 @@
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="2">
-        <v>10.8596</v>
+        <v>1</v>
       </c>
       <c r="B22" s="2">
         <v>10.7258</v>
@@ -707,7 +707,7 @@
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="2">
-        <v>10.801600000000001</v>
+        <v>1</v>
       </c>
       <c r="B23" s="2">
         <v>10.615500000000001</v>
@@ -721,7 +721,7 @@
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="2">
-        <v>10.9519</v>
+        <v>0</v>
       </c>
       <c r="B24" s="2">
         <v>10.7012</v>
@@ -735,7 +735,7 @@
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="2">
-        <v>11.023999999999999</v>
+        <v>0</v>
       </c>
       <c r="B25" s="2">
         <v>10.755599999999999</v>
@@ -749,7 +749,7 @@
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="2">
-        <v>10.8118</v>
+        <v>0</v>
       </c>
       <c r="B26" s="2">
         <v>10.7507</v>
@@ -763,7 +763,7 @@
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="2">
-        <v>10.8797</v>
+        <v>1</v>
       </c>
       <c r="B27" s="2">
         <v>10.704800000000001</v>
@@ -777,7 +777,7 @@
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="2">
-        <v>11.0273</v>
+        <v>1</v>
       </c>
       <c r="B28" s="2">
         <v>10.8421</v>
@@ -791,7 +791,7 @@
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="2">
-        <v>10.9695</v>
+        <v>0</v>
       </c>
       <c r="B29" s="2">
         <v>10.6106</v>
@@ -805,7 +805,7 @@
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="2">
-        <v>11.164099999999999</v>
+        <v>0</v>
       </c>
       <c r="B30" s="2">
         <v>10.668100000000001</v>
@@ -819,7 +819,7 @@
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="2">
-        <v>11.116899999999999</v>
+        <v>0</v>
       </c>
       <c r="B31" s="2">
         <v>10.699299999999999</v>
@@ -833,7 +833,7 @@
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="2">
-        <v>10.9848</v>
+        <v>0</v>
       </c>
       <c r="B32" s="2">
         <v>10.8172</v>
@@ -847,7 +847,7 @@
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="2">
-        <v>11.149100000000001</v>
+        <v>0</v>
       </c>
       <c r="B33" s="2">
         <v>10.7874</v>
@@ -861,7 +861,7 @@
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="2">
-        <v>11.2568</v>
+        <v>0</v>
       </c>
       <c r="B34" s="2">
         <v>10.7592</v>
@@ -875,7 +875,7 @@
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="2">
-        <v>10.791700000000001</v>
+        <v>0</v>
       </c>
       <c r="B35" s="2">
         <v>10.844799999999999</v>
@@ -889,7 +889,7 @@
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="2">
-        <v>10.9397</v>
+        <v>1</v>
       </c>
       <c r="B36" s="2">
         <v>10.76</v>
@@ -903,7 +903,7 @@
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="2">
-        <v>10.988200000000001</v>
+        <v>1</v>
       </c>
       <c r="B37" s="2">
         <v>10.742800000000001</v>
@@ -917,7 +917,7 @@
     </row>
     <row r="38" spans="1:4">
       <c r="A38" s="2">
-        <v>10.7225</v>
+        <v>0</v>
       </c>
       <c r="B38" s="2">
         <v>10.489599999999999</v>
@@ -931,7 +931,7 @@
     </row>
     <row r="39" spans="1:4">
       <c r="A39" s="2">
-        <v>10.810700000000001</v>
+        <v>0</v>
       </c>
       <c r="B39" s="2">
         <v>10.446</v>
@@ -945,7 +945,7 @@
     </row>
     <row r="40" spans="1:4">
       <c r="A40" s="2">
-        <v>10.9032</v>
+        <v>0</v>
       </c>
       <c r="B40" s="2">
         <v>10.488899999999999</v>
@@ -959,7 +959,7 @@
     </row>
     <row r="41" spans="1:4">
       <c r="A41" s="2">
-        <v>10.632</v>
+        <v>0</v>
       </c>
       <c r="B41" s="2">
         <v>10.5313</v>
@@ -973,7 +973,7 @@
     </row>
     <row r="42" spans="1:4">
       <c r="A42" s="2">
-        <v>10.883599999999999</v>
+        <v>0</v>
       </c>
       <c r="B42" s="2">
         <v>10.427300000000001</v>
@@ -987,7 +987,7 @@
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="2">
-        <v>11.2332</v>
+        <v>0</v>
       </c>
       <c r="B43" s="2">
         <v>10.3116</v>
@@ -1001,7 +1001,7 @@
     </row>
     <row r="44" spans="1:4">
       <c r="A44" s="2">
-        <v>10.749499999999999</v>
+        <v>0</v>
       </c>
       <c r="B44" s="2">
         <v>10.718500000000001</v>
@@ -1015,7 +1015,7 @@
     </row>
     <row r="45" spans="1:4">
       <c r="A45" s="2">
-        <v>10.675800000000001</v>
+        <v>1</v>
       </c>
       <c r="B45" s="2">
         <v>10.546900000000001</v>
@@ -1029,7 +1029,7 @@
     </row>
     <row r="46" spans="1:4">
       <c r="A46" s="2">
-        <v>10.8881</v>
+        <v>1</v>
       </c>
       <c r="B46" s="2">
         <v>10.620699999999999</v>
@@ -1043,7 +1043,7 @@
     </row>
     <row r="47" spans="1:4">
       <c r="A47" s="2">
-        <v>10.8165</v>
+        <v>0</v>
       </c>
       <c r="B47" s="2">
         <v>10.2966</v>
@@ -1057,7 +1057,7 @@
     </row>
     <row r="48" spans="1:4">
       <c r="A48" s="2">
-        <v>10.861599999999999</v>
+        <v>0</v>
       </c>
       <c r="B48" s="2">
         <v>10.661899999999999</v>
@@ -1071,7 +1071,7 @@
     </row>
     <row r="49" spans="1:4">
       <c r="A49" s="2">
-        <v>10.800599999999999</v>
+        <v>0</v>
       </c>
       <c r="B49" s="2">
         <v>10.723000000000001</v>
@@ -1085,7 +1085,7 @@
     </row>
     <row r="50" spans="1:4">
       <c r="A50" s="2">
-        <v>10.728400000000001</v>
+        <v>0</v>
       </c>
       <c r="B50" s="2">
         <v>10.8148</v>
@@ -1099,7 +1099,7 @@
     </row>
     <row r="51" spans="1:4">
       <c r="A51" s="2">
-        <v>10.7699</v>
+        <v>1</v>
       </c>
       <c r="B51" s="2">
         <v>10.725</v>
@@ -1113,7 +1113,7 @@
     </row>
     <row r="52" spans="1:4">
       <c r="A52" s="2">
-        <v>10.8813</v>
+        <v>1</v>
       </c>
       <c r="B52" s="2">
         <v>10.7454</v>
@@ -1127,7 +1127,7 @@
     </row>
     <row r="53" spans="1:4">
       <c r="A53" s="2">
-        <v>10.9527</v>
+        <v>0</v>
       </c>
       <c r="B53" s="2">
         <v>10.420500000000001</v>
@@ -1141,7 +1141,7 @@
     </row>
     <row r="54" spans="1:4">
       <c r="A54" s="2">
-        <v>10.9481</v>
+        <v>1</v>
       </c>
       <c r="B54" s="2">
         <v>10.410399999999999</v>
@@ -1155,7 +1155,7 @@
     </row>
     <row r="55" spans="1:4">
       <c r="A55" s="2">
-        <v>11.053000000000001</v>
+        <v>1</v>
       </c>
       <c r="B55" s="2">
         <v>10.549300000000001</v>
@@ -1169,7 +1169,7 @@
     </row>
     <row r="56" spans="1:4">
       <c r="A56" s="2">
-        <v>10.9054</v>
+        <v>0</v>
       </c>
       <c r="B56" s="2">
         <v>10.6092</v>
@@ -1183,7 +1183,7 @@
     </row>
     <row r="57" spans="1:4">
       <c r="A57" s="2">
-        <v>10.9689</v>
+        <v>0</v>
       </c>
       <c r="B57" s="2">
         <v>10.786</v>
@@ -1197,7 +1197,7 @@
     </row>
     <row r="58" spans="1:4">
       <c r="A58" s="2">
-        <v>10.964</v>
+        <v>0</v>
       </c>
       <c r="B58" s="2">
         <v>10.720499999999999</v>
@@ -1211,7 +1211,7 @@
     </row>
     <row r="59" spans="1:4">
       <c r="A59" s="2">
-        <v>10.7324</v>
+        <v>0</v>
       </c>
       <c r="B59" s="2">
         <v>10.495200000000001</v>
@@ -1225,7 +1225,7 @@
     </row>
     <row r="60" spans="1:4">
       <c r="A60" s="2">
-        <v>10.8287</v>
+        <v>1</v>
       </c>
       <c r="B60" s="2">
         <v>10.442600000000001</v>
@@ -1239,7 +1239,7 @@
     </row>
     <row r="61" spans="1:4">
       <c r="A61" s="2">
-        <v>10.8446</v>
+        <v>1</v>
       </c>
       <c r="B61" s="2">
         <v>10.4366</v>
@@ -1253,7 +1253,7 @@
     </row>
     <row r="62" spans="1:4">
       <c r="A62" s="2">
-        <v>10.9422</v>
+        <v>1</v>
       </c>
       <c r="B62" s="2">
         <v>10.4621</v>
@@ -1267,7 +1267,7 @@
     </row>
     <row r="63" spans="1:4">
       <c r="A63" s="2">
-        <v>10.819100000000001</v>
+        <v>0</v>
       </c>
       <c r="B63" s="2">
         <v>10.5252</v>
@@ -1281,7 +1281,7 @@
     </row>
     <row r="64" spans="1:4">
       <c r="A64" s="2">
-        <v>10.905900000000001</v>
+        <v>0</v>
       </c>
       <c r="B64" s="2">
         <v>10.6221</v>

</xml_diff>